<commit_message>
automate until user role dynamic dropdown
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12300"/>
+    <workbookView windowWidth="27945" windowHeight="11850"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -27,15 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Username</t>
   </si>
   <si>
     <t>Password</t>
-  </si>
-  <si>
-    <t>ExpectedResult</t>
   </si>
   <si>
     <t>Admin</t>
@@ -44,13 +41,16 @@
     <t>admin123</t>
   </si>
   <si>
-    <t>Success</t>
+    <t>user1</t>
   </si>
   <si>
-    <t>wrongpwd</t>
+    <t>pass123</t>
   </si>
   <si>
-    <t>Failure</t>
+    <t>user2</t>
+  </si>
+  <si>
+    <t>pass456</t>
   </si>
 </sst>
 </file>
@@ -674,12 +674,18 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1217,8 +1223,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="2"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" ht="30" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -1227,29 +1233,31 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" ht="30" spans="1:3">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" ht="30" spans="1:3">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="C3" s="4"/>
     </row>
-    <row r="3" ht="30" spans="1:3">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="4" spans="1:2">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>